<commit_message>
feat: add construction planning, Project exchange and site routing
</commit_message>
<xml_diff>
--- a/docs/civil-buddy/open-source-integrate.xlsx
+++ b/docs/civil-buddy/open-source-integrate.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="建议接入" sheetId="1" r:id="R31d270d2396b4b71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="不要并仓" sheetId="2" r:id="Rd8d6714b367a407f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GitHub加深检索" sheetId="3" r:id="Re37da71e41a043d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核验候选" sheetId="4" r:id="R9925e9506dcd476a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="比赛交付" sheetId="5" r:id="Rfa5454ab0e724c80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GitHub加深命中" sheetId="6" r:id="R9a9236e642b14be9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="建议接入" sheetId="1" r:id="R1d3c4cdc4a8a40d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="不要并仓" sheetId="2" r:id="R21ba54d98c8f4515"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GitHub加深检索" sheetId="3" r:id="R4a081bc892434b02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核验候选" sheetId="4" r:id="R1a18e6dc08d341e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="比赛交付" sheetId="5" r:id="R1c8c8393ae774a60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GitHub加深命中" sheetId="6" r:id="R304713a105d54dd0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -119,7 +119,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="28">
+  <x:cellXfs count="31">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -192,11 +192,18 @@
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="2">
+  <x:dxfs count="3">
     <x:dxf>
       <x:font>
         <x:color rgb="FF7F6000"/>
@@ -213,6 +220,13 @@
       </x:font>
       <x:fill>
         <x:patternFill>
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -318,7 +332,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="VerifiedCandidates" displayName="VerifiedCandidates" ref="A1:S15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="VerifiedCandidates" displayName="VerifiedCandidates" ref="A1:S21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="19">
     <x:tableColumn id="1" name="编号"/>
     <x:tableColumn id="2" name="项目"/>
@@ -1768,7 +1782,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14b581b24b534e76"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd49a6a213cb74341"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2326,7 +2340,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15fc5f9cbad640ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b6384eb213d48fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2838,25 +2852,19 @@
           <x:t xml:space="preserve">P0 首批</x:t>
         </x:is>
       </x:c>
-      <x:c r="D4" s="16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">施工计划编辑</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E4" s="16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">拖动任务日期、调整完成率和查看前后置关系，接入保存与撤销。</x:t>
-        </x:is>
+      <x:c r="D4" s="16" t="str">
+        <x:v>日期甘特与排程结果展示</x:v>
+      </x:c>
+      <x:c r="E4" s="16" t="str">
+        <x:v>保留日期/进度拖动与撤销；新排程页展示自研CPM和资源方案。</x:v>
       </x:c>
       <x:c r="F4" s="16" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">plan-master / plan-lookahead</x:t>
         </x:is>
       </x:c>
-      <x:c r="G4" s="16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">本地 JS 控件，date_change/progress_change 回写后端。</x:t>
-        </x:is>
+      <x:c r="G4" s="16" t="str">
+        <x:v>本地1.2.2控件；日期页可编辑，排程页只读图配参数编辑。</x:v>
       </x:c>
       <x:c r="H4" s="16" t="inlineStr">
         <x:is>
@@ -2869,22 +2877,18 @@
         </x:is>
       </x:c>
       <x:c r="J4" s="16" t="str">
-        <x:v>已接入；离线与 HTTP 通过；浏览器拖动/撤销/保存刷新/390px 通过；真实项目待验收</x:v>
+        <x:v>已接入；拖动/撤销/重开通过；新排程页390px通过；真实计划待验。</x:v>
       </x:c>
       <x:c r="K4" s="16" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">任务名称、日期、依赖及完成率；未填日期不自动假造工期。</x:t>
         </x:is>
       </x:c>
-      <x:c r="L4" s="16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">修改任务后保存重开一致，撤销可还原，循环依赖被拒绝。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M4" s="16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">是甘特编辑控件，不自带完整 CPM、资源平衡或施工日历求解。</x:t>
-        </x:is>
+      <x:c r="L4" s="16" t="str">
+        <x:v>旧日期手势可一次撤销；新页CPM8天/资源11天、保存重启恢复。</x:v>
+      </x:c>
+      <x:c r="M4" s="16" t="str">
+        <x:v>控件负责显示与日期编辑；CPM/资源求解来自本项目内核及OR-Tools。</x:v>
       </x:c>
       <x:c r="N4" s="16" t="str">
         <x:v>本轮采用 npm 1.2.2；官方 tarball 完整性及许可见 vendor/SOURCE.json。早期 GitHub release 记录 v1.0.3。</x:v>
@@ -3939,6 +3943,358 @@
       <x:c r="Q15" s="16" t="str"/>
       <x:c r="R15" s="16" t="str"/>
       <x:c r="S15" s="25" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="90" customHeight="1">
+      <x:c r="A16" s="27" t="str">
+        <x:v>N15</x:v>
+      </x:c>
+      <x:c r="B16" s="27" t="str">
+        <x:v>Civil Buddy CPM / 基线 / 周 PPC</x:v>
+      </x:c>
+      <x:c r="C16" s="27" t="str">
+        <x:v>P0 深化</x:v>
+      </x:c>
+      <x:c r="D16" s="27" t="str">
+        <x:v>施工排程与进度管理</x:v>
+      </x:c>
+      <x:c r="E16" s="27" t="str">
+        <x:v>工作日历、WBS、四类依赖、正负时距、关键任务、基线与周承诺。</x:v>
+      </x:c>
+      <x:c r="F16" s="27" t="str">
+        <x:v>plan-master / plan-lookahead</x:v>
+      </x:c>
+      <x:c r="G16" s="27" t="str">
+        <x:v>本项目 Python 内核和版本存储；Frappe 展示计算结果。</x:v>
+      </x:c>
+      <x:c r="H16" s="27" t="str">
+        <x:v>本项目 MIT；前端及求解器依赖分别署名。</x:v>
+      </x:c>
+      <x:c r="I16" s="27" t="str">
+        <x:v>说明自研范围，保留明确输入、结果版本与测试证据。</x:v>
+      </x:c>
+      <x:c r="J16" s="27" t="str">
+        <x:v>已接入；核心15项、HTTP14项；浏览器真重启恢复资源11天。</x:v>
+      </x:c>
+      <x:c r="K16" s="27" t="str">
+        <x:v>明确工期、工作日历、依赖、完成事实；不从名称猜工期。</x:v>
+      </x:c>
+      <x:c r="L16" s="27" t="str">
+        <x:v>合成 CPM 8天；基线8天、资源11天、PPC50%；重开一致。</x:v>
+      </x:c>
+      <x:c r="M16" s="27" t="str">
+        <x:v>统一日历、整工作日；实际日期仅记录；不是完整 MSP/P6 引擎。</x:v>
+      </x:c>
+      <x:c r="N16" s="27" t="str">
+        <x:v>本轮本地实现及离线、HTTP、浏览器记录。</x:v>
+      </x:c>
+      <x:c r="O16" s="27" t="str">
+        <x:v>https://github.com/LUOaini1213/civil-buddy</x:v>
+      </x:c>
+      <x:c r="P16" s="27" t="str">
+        <x:v>docs/civil-buddy/planning-workbench.md</x:v>
+      </x:c>
+      <x:c r="Q16" s="27" t="str">
+        <x:v>https://github.com/LUOaini1213/civil-buddy/blob/main/LICENSE</x:v>
+      </x:c>
+      <x:c r="R16" s="27" t="str">
+        <x:v>本轮变更在工作分支，公开默认分支可能尚未同步。</x:v>
+      </x:c>
+      <x:c r="S16" s="30" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="90" customHeight="1">
+      <x:c r="A17" s="27" t="str">
+        <x:v>N16</x:v>
+      </x:c>
+      <x:c r="B17" s="27" t="str">
+        <x:v>OR-Tools CP-SAT</x:v>
+      </x:c>
+      <x:c r="C17" s="27" t="str">
+        <x:v>P0 深化</x:v>
+      </x:c>
+      <x:c r="D17" s="27" t="str">
+        <x:v>资源容量约束排程</x:v>
+      </x:c>
+      <x:c r="E17" s="27" t="str">
+        <x:v>明确班组/设备容量下求可行或最优日期，预览后应用，可撤销。</x:v>
+      </x:c>
+      <x:c r="F17" s="27" t="str">
+        <x:v>plan-resource / plan-master</x:v>
+      </x:c>
+      <x:c r="G17" s="27" t="str">
+        <x:v>固定 Python worker；区间与累计资源约束；不执行模型代码。</x:v>
+      </x:c>
+      <x:c r="H17" s="27" t="str">
+        <x:v>Apache-2.0；传递依赖保留各自许可。</x:v>
+      </x:c>
+      <x:c r="I17" s="27" t="str">
+        <x:v>保留版本、LICENSE 与适用 NOTICE；区分自研适配和求解器。</x:v>
+      </x:c>
+      <x:c r="J17" s="27" t="str">
+        <x:v>已接入；优化9项；单班组11天、双班组8天通过。</x:v>
+      </x:c>
+      <x:c r="K17" s="27" t="str">
+        <x:v>整数工期、四类依赖、资源容量及工序明确需求。</x:v>
+      </x:c>
+      <x:c r="L17" s="27" t="str">
+        <x:v>CPM8天→单班组11天→保存重启恢复；进度改动不静默降级。</x:v>
+      </x:c>
+      <x:c r="M17" s="27" t="str">
+        <x:v>统一日历、不可中断、整单位资源；OPTIMAL才证明最优；不算资源关键线路。</x:v>
+      </x:c>
+      <x:c r="N17" s="27" t="str">
+        <x:v>已安装锁定 ortools 9.15.6755，实际求解通过。</x:v>
+      </x:c>
+      <x:c r="O17" s="27" t="str">
+        <x:v>https://github.com/google/or-tools</x:v>
+      </x:c>
+      <x:c r="P17" s="27" t="str">
+        <x:v>https://developers.google.com/optimization/scheduling/job_shop</x:v>
+      </x:c>
+      <x:c r="Q17" s="27" t="str">
+        <x:v>https://github.com/google/or-tools/blob/v9.15/LICENSE</x:v>
+      </x:c>
+      <x:c r="R17" s="27" t="str">
+        <x:v>https://developers.google.com/optimization/cp/cp_solver</x:v>
+      </x:c>
+      <x:c r="S17" s="30" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="90" customHeight="1">
+      <x:c r="A18" s="27" t="str">
+        <x:v>N17</x:v>
+      </x:c>
+      <x:c r="B18" s="27" t="str">
+        <x:v>MPXJ</x:v>
+      </x:c>
+      <x:c r="C18" s="27" t="str">
+        <x:v>P0 深化</x:v>
+      </x:c>
+      <x:c r="D18" s="27" t="str">
+        <x:v>MPP / P6 计划文件读取</x:v>
+      </x:c>
+      <x:c r="E18" s="27" t="str">
+        <x:v>MPP、XER、PMXML 转受限 MSPDI；展示原日期与未映射报告，确认后应用。</x:v>
+      </x:c>
+      <x:c r="F18" s="27" t="str">
+        <x:v>plan-master / 文件导入</x:v>
+      </x:c>
+      <x:c r="G18" s="27" t="str">
+        <x:v>MPXJ 16.7.0 + JPype1 1.7.1 + 便携 JRE21，固定子进程。</x:v>
+      </x:c>
+      <x:c r="H18" s="27" t="str">
+        <x:v>LGPL-2.1；JPype、JRE 与捆绑 Java 库另按各自条款。</x:v>
+      </x:c>
+      <x:c r="I18" s="27" t="str">
+        <x:v>保留准确版本许可、来源与摘要；分发时核对 LGPL 和捆绑库要求。</x:v>
+      </x:c>
+      <x:c r="J18" s="27" t="str">
+        <x:v>已接入；公开MPP16任务网页上传/保存刷新通过；P6合成往返通过。</x:v>
+      </x:c>
+      <x:c r="K18" s="27" t="str">
+        <x:v>单项目文件，明确日历/工期；另行保存授权原始文件。</x:v>
+      </x:c>
+      <x:c r="L18" s="27" t="str">
+        <x:v>二进制MPP读入16任务/16原日期；XER/PMXML实际读取。</x:v>
+      </x:c>
+      <x:c r="M18" s="27" t="str">
+        <x:v>不写原生MPP/P6；不等于源排程引擎；部分资源占用明确拒绝。</x:v>
+      </x:c>
+      <x:c r="N18" s="27" t="str">
+        <x:v>锁定 mpxj16.7.0；官方MPP固定提交文件与SHA256已核验。</x:v>
+      </x:c>
+      <x:c r="O18" s="27" t="str">
+        <x:v>https://github.com/joniles/mpxj</x:v>
+      </x:c>
+      <x:c r="P18" s="27" t="str">
+        <x:v>https://www.mpxj.org/</x:v>
+      </x:c>
+      <x:c r="Q18" s="27" t="str">
+        <x:v>https://github.com/joniles/mpxj/blob/v16.7.0/LICENSE</x:v>
+      </x:c>
+      <x:c r="R18" s="27" t="str">
+        <x:v>https://github.com/joniles/mpxj/blob/c5e1320cde0acd404031495aa66c17639a57239b/junit/data/generated/task-links/task-links-project2000-mpp9.mpp</x:v>
+      </x:c>
+      <x:c r="S18" s="30" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="90" customHeight="1">
+      <x:c r="A19" s="27" t="str">
+        <x:v>N18</x:v>
+      </x:c>
+      <x:c r="B19" s="27" t="str">
+        <x:v>NetworkX</x:v>
+      </x:c>
+      <x:c r="C19" s="27" t="str">
+        <x:v>P0 深化</x:v>
+      </x:c>
+      <x:c r="D19" s="27" t="str">
+        <x:v>场内最短路线</x:v>
+      </x:c>
+      <x:c r="E19" s="27" t="str">
+        <x:v>编辑明确道路权重、方向和封路状态，显示最短路线及分段来源。</x:v>
+      </x:c>
+      <x:c r="F19" s="27" t="str">
+        <x:v>dispatch / municipal / routes</x:v>
+      </x:c>
+      <x:c r="G19" s="27" t="str">
+        <x:v>Python MultiDiGraph + Dijkstra，独立道路页面。</x:v>
+      </x:c>
+      <x:c r="H19" s="27" t="str">
+        <x:v>BSD-3-Clause。</x:v>
+      </x:c>
+      <x:c r="I19" s="27" t="str">
+        <x:v>保留版权、许可与版本；道路数据授权单独确认。</x:v>
+      </x:c>
+      <x:c r="J19" s="27" t="str">
+        <x:v>已接入；路线8项；桌面浏览器150m→封路180m→不可达。</x:v>
+      </x:c>
+      <x:c r="K19" s="27" t="str">
+        <x:v>道路节点和每段明确距离(m)或固定通行时间(min)、数值来源。</x:v>
+      </x:c>
+      <x:c r="L19" s="27" t="str">
+        <x:v>单向/封路/不可达；平行边来源和单位核对。</x:v>
+      </x:c>
+      <x:c r="M19" s="27" t="str">
+        <x:v>道路最短路不是施工CPM；不猜车速，不做车辆调度；未接独立项目保存。</x:v>
+      </x:c>
+      <x:c r="N19" s="27" t="str">
+        <x:v>已安装锁定 networkx3.6.1；实际算法与页面验证通过。</x:v>
+      </x:c>
+      <x:c r="O19" s="27" t="str">
+        <x:v>https://github.com/networkx/networkx</x:v>
+      </x:c>
+      <x:c r="P19" s="27" t="str">
+        <x:v>https://networkx.org/documentation/stable/reference/algorithms/shortest_paths.html</x:v>
+      </x:c>
+      <x:c r="Q19" s="27" t="str">
+        <x:v>https://github.com/networkx/networkx/blob/networkx-3.6.1/LICENSE.txt</x:v>
+      </x:c>
+      <x:c r="R19" s="27" t="str">
+        <x:v>https://networkx.org/documentation/stable/reference/classes/multidigraph.html</x:v>
+      </x:c>
+      <x:c r="S19" s="30" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="90" customHeight="1">
+      <x:c r="A20" s="27" t="str">
+        <x:v>N19</x:v>
+      </x:c>
+      <x:c r="B20" s="27" t="str">
+        <x:v>OpenProject</x:v>
+      </x:c>
+      <x:c r="C20" s="27" t="str">
+        <x:v>P2 后续</x:v>
+      </x:c>
+      <x:c r="D20" s="27" t="str">
+        <x:v>项目协作平台候选</x:v>
+      </x:c>
+      <x:c r="E20" s="27" t="str">
+        <x:v>候选方向：多人工作包、责任人与项目协作；先做独立接口验证。</x:v>
+      </x:c>
+      <x:c r="F20" s="27" t="str">
+        <x:v>plan-master / 协作候选</x:v>
+      </x:c>
+      <x:c r="G20" s="27" t="str">
+        <x:v>尚未接入；后续评估官方API与部署，不嵌入整套平台。</x:v>
+      </x:c>
+      <x:c r="H20" s="27" t="str">
+        <x:v>官方主仓 LICENSE 为 GPLv3；选版及扩展功能另核。</x:v>
+      </x:c>
+      <x:c r="I20" s="27" t="str">
+        <x:v>采用前锁定版本及实际部署/复制范围，保留源码与许可证义务。</x:v>
+      </x:c>
+      <x:c r="J20" s="27" t="str">
+        <x:v>后续候选，未安装、未接入、未验收。</x:v>
+      </x:c>
+      <x:c r="K20" s="27" t="str">
+        <x:v>测试项目、用户/权限边界、实际协作需求。</x:v>
+      </x:c>
+      <x:c r="L20" s="27" t="str">
+        <x:v>采用前验证工作包读取/更新、权限、冲突与审计。</x:v>
+      </x:c>
+      <x:c r="M20" s="27" t="str">
+        <x:v>不将平台宣传等同当前工作台能力，不声称 Project/P6 无损互通。</x:v>
+      </x:c>
+      <x:c r="N20" s="27" t="str">
+        <x:v>本轮只核官方仓库/许可入口；版本、维护及API验证待补。</x:v>
+      </x:c>
+      <x:c r="O20" s="27" t="str">
+        <x:v>https://github.com/opf/openproject</x:v>
+      </x:c>
+      <x:c r="P20" s="27" t="str">
+        <x:v>https://www.openproject.org/docs/api/</x:v>
+      </x:c>
+      <x:c r="Q20" s="27" t="str">
+        <x:v>https://github.com/opf/openproject/blob/dev/LICENSE</x:v>
+      </x:c>
+      <x:c r="R20" s="27" t="str">
+        <x:v>https://www.openproject.org/docs/</x:v>
+      </x:c>
+      <x:c r="S20" s="30" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="90" customHeight="1">
+      <x:c r="A21" s="27" t="str">
+        <x:v>N20</x:v>
+      </x:c>
+      <x:c r="B21" s="27" t="str">
+        <x:v>GanttProject</x:v>
+      </x:c>
+      <x:c r="C21" s="27" t="str">
+        <x:v>P3 备选</x:v>
+      </x:c>
+      <x:c r="D21" s="27" t="str">
+        <x:v>桌面计划与互通候选</x:v>
+      </x:c>
+      <x:c r="E21" s="27" t="str">
+        <x:v>候选方向：桌面甘特流程参考与文件交换对照。</x:v>
+      </x:c>
+      <x:c r="F21" s="27" t="str">
+        <x:v>plan-master / 互通候选</x:v>
+      </x:c>
+      <x:c r="G21" s="27" t="str">
+        <x:v>尚未接入；先核文件往返与可调用接口，不复制整套桌面应用。</x:v>
+      </x:c>
+      <x:c r="H21" s="27" t="str">
+        <x:v>官方主仓 LICENSE 为 GPLv3；分发组件逐项核对。</x:v>
+      </x:c>
+      <x:c r="I21" s="27" t="str">
+        <x:v>采用前锁定版本及复制范围，保留许可、版权和对应源码要求。</x:v>
+      </x:c>
+      <x:c r="J21" s="27" t="str">
+        <x:v>后续候选，未安装、未接入、未验收。</x:v>
+      </x:c>
+      <x:c r="K21" s="27" t="str">
+        <x:v>授权计划文件、明确工期/日历/资源，源软件对照结果。</x:v>
+      </x:c>
+      <x:c r="L21" s="27" t="str">
+        <x:v>采用前验证实际日期、依赖、WBS和资源往返差异。</x:v>
+      </x:c>
+      <x:c r="M21" s="27" t="str">
+        <x:v>不能据README声称已兼容全部MSP/P6；当前主线仍为自研受限排程。</x:v>
+      </x:c>
+      <x:c r="N21" s="27" t="str">
+        <x:v>本轮只核官方仓库/许可入口；具体版本能力待验证。</x:v>
+      </x:c>
+      <x:c r="O21" s="27" t="str">
+        <x:v>https://github.com/bardsoftware/ganttproject</x:v>
+      </x:c>
+      <x:c r="P21" s="27" t="str">
+        <x:v>https://www.ganttproject.biz/</x:v>
+      </x:c>
+      <x:c r="Q21" s="27" t="str">
+        <x:v>https://github.com/bardsoftware/ganttproject/blob/master/LICENSE</x:v>
+      </x:c>
+      <x:c r="R21" s="27"/>
+      <x:c r="S21" s="30" t="n">
         <x:v>46286</x:v>
       </x:c>
     </x:row>
@@ -3947,14 +4303,20 @@
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="尚待集成验收"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="已集成验收"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="1">
+  <x:conditionalFormatting sqref="J16:J21">
+    <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="已接入"/>
+  </x:conditionalFormatting>
+  <x:dataValidations count="2">
     <x:dataValidation type="list" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C2:C15">
       <x:formula1>"P0 首批,P1 后续,P2 后续,P3 备选,P3 暂缓"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="C16:C21">
+      <x:formula1>"P0 深化,P1 后续,P2 后续,P3 备选,P3 暂缓"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc3b8967dfc240e8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc70dec6a42f4d85"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4006,15 +4368,15 @@
         </x:is>
       </x:c>
       <x:c r="D3" s="16" t="n">
-        <x:f>COUNTIFS('核验候选'!$C$2:$C$15,"P0 首批")</x:f>
+        <x:f>COUNTIFS('核验候选'!$C$2:$C$21,"P0 首批")</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="E3" s="16" t="str">
         <x:v>主清单记录数（含历史）</x:v>
       </x:c>
       <x:c r="F3" s="16" t="n">
-        <x:f>COUNTA('建议接入'!$B$5:$B$22)+COUNTA('不要并仓'!$A$5:$A$17)+COUNTA('核验候选'!$B$2:$B$15)</x:f>
-        <x:v>45</x:v>
+        <x:f>COUNTA('建议接入'!$B$5:$B$22)+COUNTA('不要并仓'!$A$5:$A$17)+COUNTA('核验候选'!$B$2:$B$21)</x:f>
+        <x:v>51</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -4123,28 +4485,20 @@
           <x:t xml:space="preserve">首批 3</x:t>
         </x:is>
       </x:c>
-      <x:c r="B8" s="16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">施工甘特</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C8" s="16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">添加任务与依赖 → 改日期 → 保存 → 重开 → 撤销</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D8" s="16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">任务计划由参赛团队录入</x:t>
-        </x:is>
+      <x:c r="B8" s="16" t="str">
+        <x:v>施工排程与日期甘特</x:v>
+      </x:c>
+      <x:c r="C8" s="16" t="str">
+        <x:v>明确工期/日历→CPM→资源预览→保存重启恢复→基线/周PPC</x:v>
+      </x:c>
+      <x:c r="D8" s="16" t="str">
+        <x:v>团队录入明确任务、日历和整单位资源；真实计划尚未提供。</x:v>
       </x:c>
       <x:c r="E8" s="16" t="str">
-        <x:v>已接入；离线与 HTTP 通过；浏览器拖动/撤销/保存刷新/390px 通过；真实项目待验收</x:v>
-      </x:c>
-      <x:c r="F8" s="16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Frappe Gantt，首版无完整 CPM</x:t>
-        </x:is>
+        <x:v>已接入；CPM8天、资源11天、基线8天、PPC50%；重启与390px通过。</x:v>
+      </x:c>
+      <x:c r="F8" s="16" t="str">
+        <x:v>Frappe Gantt + 自研CPM/版本/PPC + OR-Tools；文件读取MPXJ。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="60" customHeight="1">
@@ -4241,13 +4595,25 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="16" t="n"/>
-      <x:c r="B12" s="16" t="n"/>
-      <x:c r="C12" s="16" t="n"/>
-      <x:c r="D12" s="16" t="n"/>
-      <x:c r="E12" s="16" t="n"/>
-      <x:c r="F12" s="16" t="n"/>
+    <x:row r="12" ht="60" customHeight="1">
+      <x:c r="A12" s="16" t="str">
+        <x:v>本轮深化</x:v>
+      </x:c>
+      <x:c r="B12" s="16" t="str">
+        <x:v>场内最短路线</x:v>
+      </x:c>
+      <x:c r="C12" s="16" t="str">
+        <x:v>明确道路→150m→封路180m→不可达</x:v>
+      </x:c>
+      <x:c r="D12" s="16" t="str">
+        <x:v>节点、单向/双向、封路和距离/时间来源</x:v>
+      </x:c>
+      <x:c r="E12" s="16" t="str">
+        <x:v>已接入；离线8项与桌面浏览器通过；真实路网待验。</x:v>
+      </x:c>
+      <x:c r="F12" s="16" t="str">
+        <x:v>NetworkX，独立于施工关键路径。</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="16" t="n"/>
@@ -4359,20 +4725,16 @@
           <x:t xml:space="preserve">同事 C / 计划与演示</x:t>
         </x:is>
       </x:c>
-      <x:c r="B18" s="16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Frappe 甘特、任务编辑、日期/依赖校验、截图与比赛材料</x:t>
-        </x:is>
+      <x:c r="B18" s="16" t="str">
+        <x:v>施工日历/依赖、资源方案、基线周PPC、文件往返与比赛材料</x:v>
       </x:c>
       <x:c r="C18" s="16" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">沿用项目存储和撤销，不另起第二套业务后台</x:t>
         </x:is>
       </x:c>
-      <x:c r="D18" s="16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">计划改动保存重开一致；演示视频区分自研和复用</x:t>
-        </x:is>
+      <x:c r="D18" s="16" t="str">
+        <x:v>8/11天算例、MPP/P6读取、重启恢复；区分自研与复用、真实与合成。</x:v>
       </x:c>
       <x:c r="E18" s="16" t="n"/>
       <x:c r="F18" s="16" t="n"/>
@@ -4438,7 +4800,7 @@
         </x:is>
       </x:c>
       <x:c r="B24" s="16" t="str">
-        <x:v>保留全部当前 6 张表，包括后续补入的 8 条主表记录和 15 条检索命中。第 6 表多为重复来源，不重复计入主清单。</x:v>
+        <x:v>保留全部6张表与历史记录，追加本轮6项排程/路线/候选。第6表15条检索命中不重复计数。</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="40" customHeight="1">
@@ -4602,44 +4964,60 @@
         <x:v>数量口径</x:v>
       </x:c>
       <x:c r="B39" s="27" t="str">
-        <x:v>45 条为 18 条建议、13 条历史暂缓、14 条本轮新增/深化记录，含书签与同生态功能；不是 45 个独立项目。15 条检索命中不重复计数。</x:v>
+        <x:v>51条为18条建议、13条历史暂缓、20条新增/深化，含自研模块、组件及书签，不是51个独立开源项目。15条检索命中不重复计数。</x:v>
       </x:c>
       <x:c r="C39" s="27" t="n"/>
       <x:c r="D39" s="27" t="n"/>
       <x:c r="E39" s="27" t="n"/>
       <x:c r="F39" s="27" t="n"/>
     </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="16" t="n"/>
-      <x:c r="B40" s="16" t="n"/>
-      <x:c r="C40" s="16" t="n"/>
-      <x:c r="D40" s="16" t="n"/>
-      <x:c r="E40" s="16" t="n"/>
-      <x:c r="F40" s="16" t="n"/>
-    </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="16" t="n"/>
-      <x:c r="B41" s="16" t="n"/>
-      <x:c r="C41" s="16" t="n"/>
-      <x:c r="D41" s="16" t="n"/>
-      <x:c r="E41" s="16" t="n"/>
-      <x:c r="F41" s="16" t="n"/>
-    </x:row>
-    <x:row r="42">
-      <x:c r="A42" s="16" t="n"/>
-      <x:c r="B42" s="16" t="n"/>
-      <x:c r="C42" s="16" t="n"/>
-      <x:c r="D42" s="16" t="n"/>
-      <x:c r="E42" s="16" t="n"/>
-      <x:c r="F42" s="16" t="n"/>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="16" t="n"/>
-      <x:c r="B43" s="16" t="n"/>
-      <x:c r="C43" s="16" t="n"/>
-      <x:c r="D43" s="16" t="n"/>
-      <x:c r="E43" s="16" t="n"/>
-      <x:c r="F43" s="16" t="n"/>
+    <x:row r="40" ht="54" customHeight="1">
+      <x:c r="A40" s="16" t="str">
+        <x:v>本轮排程验收</x:v>
+      </x:c>
+      <x:c r="B40" s="16" t="str">
+        <x:v>最终npm check 108/108；提交边界专项3/3；核心15、优化9、交换19、路线8、UI18、HTTP14通过。浏览器资源11天重启仍11，基线8天，PPC50%。390px仅排程页；路线桌面验收。</x:v>
+      </x:c>
+      <x:c r="C40" s="16"/>
+      <x:c r="D40" s="16"/>
+      <x:c r="E40" s="16"/>
+      <x:c r="F40" s="16"/>
+    </x:row>
+    <x:row r="41" ht="54" customHeight="1">
+      <x:c r="A41" s="16" t="str">
+        <x:v>计划文件交接</x:v>
+      </x:c>
+      <x:c r="B41" s="16" t="str">
+        <x:v>MPP公开合成文件16任务/16原日期，网页上传确认后保存刷新恢复。P6为合成XER/PMXML往返。JSON是计划交换文件，不含基线/周承诺/历史/原文件字节，非完整项目包。</x:v>
+      </x:c>
+      <x:c r="C41" s="16"/>
+      <x:c r="D41" s="16"/>
+      <x:c r="E41" s="16"/>
+      <x:c r="F41" s="16"/>
+    </x:row>
+    <x:row r="42" ht="54" customHeight="1">
+      <x:c r="A42" s="16" t="str">
+        <x:v>实现与候选边界</x:v>
+      </x:c>
+      <x:c r="B42" s="16" t="str">
+        <x:v>Frappe、自研CPM/基线周PPC、OR-Tools、MPXJ、NetworkX已接入。OpenProject/GanttProject仍为后续候选。资源仅整单位，1对应XML1.0；50%占用拒绝。真实计划未提供。</x:v>
+      </x:c>
+      <x:c r="C42" s="16"/>
+      <x:c r="D42" s="16"/>
+      <x:c r="E42" s="16"/>
+      <x:c r="F42" s="16"/>
+    </x:row>
+    <x:row r="43" ht="54" customHeight="1">
+      <x:c r="A43" s="16" t="str">
+        <x:v>部署与证据</x:v>
+      </x:c>
+      <x:c r="B43" s="16" t="str">
+        <x:v>详见 docs/civil-buddy/planning-workbench.md。MPXJ使用项目本地便携JRE，不装系统Java；保留SHA256与许可。源Project/P6软件重开、跨电脑迁移及真实施工验收仍待补。</x:v>
+      </x:c>
+      <x:c r="C43" s="16"/>
+      <x:c r="D43" s="16"/>
+      <x:c r="E43" s="16"/>
+      <x:c r="F43" s="16"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="16" t="n"/>
@@ -4667,6 +5045,10 @@
     <x:mergeCell ref="B27:F27"/>
     <x:mergeCell ref="B38:F38"/>
     <x:mergeCell ref="B39:F39"/>
+    <x:mergeCell ref="B40:F40"/>
+    <x:mergeCell ref="B41:F41"/>
+    <x:mergeCell ref="B42:F42"/>
+    <x:mergeCell ref="B43:F43"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>